<commit_message>
A single /uploads needed to be changed in to the /SBMuploads. i have done that.
</commit_message>
<xml_diff>
--- a/SBM/data.xlsx
+++ b/SBM/data.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="27">
   <si>
     <t>Apurve Srivastava</t>
   </si>
@@ -29,28 +29,34 @@
     <t>6-A ACHARYA KRIPLANI MARG NEAR MOTI</t>
   </si>
   <si>
-    <t>jgBBFtwz</t>
+    <t>MK4APzB4</t>
+  </si>
+  <si>
+    <t>["New Release","Catalogue"]</t>
+  </si>
+  <si>
+    <t>["Cntent ID Request","Artist channel Request"]</t>
+  </si>
+  <si>
+    <t>Test user</t>
+  </si>
+  <si>
+    <t>test2@gmail.com</t>
+  </si>
+  <si>
+    <t>01234567890</t>
+  </si>
+  <si>
+    <t>sdfsfs</t>
+  </si>
+  <si>
+    <t>UkifGub1</t>
   </si>
   <si>
     <t>["New Release","Catalogue","Payment"]</t>
   </si>
   <si>
     <t>["Claim Release","Cntent ID Request","Artist channel Request"]</t>
-  </si>
-  <si>
-    <t>Test user</t>
-  </si>
-  <si>
-    <t>test2@gmail.com</t>
-  </si>
-  <si>
-    <t>01234567890</t>
-  </si>
-  <si>
-    <t>sdfsfs</t>
-  </si>
-  <si>
-    <t>UkifGub1</t>
   </si>
   <si>
     <t>test5@gmail.com</t>
@@ -493,10 +499,10 @@
         <v>11</v>
       </c>
       <c r="F2" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="G2" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -504,7 +510,7 @@
         <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C3" t="s">
         <v>9</v>
@@ -513,13 +519,13 @@
         <v>10</v>
       </c>
       <c r="E3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" t="s">
         <v>13</v>
-      </c>
-      <c r="F3" t="s">
-        <v>5</v>
-      </c>
-      <c r="G3" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -527,7 +533,7 @@
         <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C4" t="s">
         <v>9</v>
@@ -536,10 +542,10 @@
         <v>10</v>
       </c>
       <c r="E4" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F4" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -547,7 +553,7 @@
         <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C5" t="s">
         <v>9</v>
@@ -556,10 +562,10 @@
         <v>10</v>
       </c>
       <c r="E5" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F5" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -567,7 +573,7 @@
         <v>7</v>
       </c>
       <c r="B6" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C6" t="s">
         <v>9</v>
@@ -576,10 +582,10 @@
         <v>10</v>
       </c>
       <c r="E6" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F6" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -598,42 +604,42 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B3" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B4" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B5" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
in SBM Digital Edit User button click genrating error in its related routes I have resolved it now its working properly
</commit_message>
<xml_diff>
--- a/SBM/data.xlsx
+++ b/SBM/data.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="25">
   <si>
     <t>Apurve Srivastava</t>
   </si>
@@ -29,13 +29,13 @@
     <t>6-A ACHARYA KRIPLANI MARG NEAR MOTI</t>
   </si>
   <si>
-    <t>MK4APzB4</t>
-  </si>
-  <si>
-    <t>["New Release","Catalogue"]</t>
-  </si>
-  <si>
-    <t>["Cntent ID Request","Artist channel Request"]</t>
+    <t>3EFFVBw9</t>
+  </si>
+  <si>
+    <t>["New Release","Catalogue","Payment"]</t>
+  </si>
+  <si>
+    <t>["Claim Release","Cntent ID Request","Artist channel Request"]</t>
   </si>
   <si>
     <t>Test user</t>
@@ -51,12 +51,6 @@
   </si>
   <si>
     <t>UkifGub1</t>
-  </si>
-  <si>
-    <t>["New Release","Catalogue","Payment"]</t>
-  </si>
-  <si>
-    <t>["Claim Release","Cntent ID Request","Artist channel Request"]</t>
   </si>
   <si>
     <t>test5@gmail.com</t>
@@ -499,10 +493,10 @@
         <v>11</v>
       </c>
       <c r="F2" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="G2" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -510,7 +504,7 @@
         <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C3" t="s">
         <v>9</v>
@@ -519,13 +513,13 @@
         <v>10</v>
       </c>
       <c r="E3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F3" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="G3" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -533,7 +527,7 @@
         <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C4" t="s">
         <v>9</v>
@@ -542,10 +536,10 @@
         <v>10</v>
       </c>
       <c r="E4" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F4" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -553,7 +547,7 @@
         <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C5" t="s">
         <v>9</v>
@@ -562,10 +556,10 @@
         <v>10</v>
       </c>
       <c r="E5" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F5" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -573,7 +567,7 @@
         <v>7</v>
       </c>
       <c r="B6" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C6" t="s">
         <v>9</v>
@@ -582,10 +576,10 @@
         <v>10</v>
       </c>
       <c r="E6" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F6" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -604,42 +598,42 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B3" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" t="s">
         <v>23</v>
-      </c>
-      <c r="B4" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
I have added new Build for the Apurve repo
</commit_message>
<xml_diff>
--- a/SBM/data.xlsx
+++ b/SBM/data.xlsx
@@ -20,16 +20,16 @@
     <t>Apurve Srivastava</t>
   </si>
   <si>
-    <t>apurve2013@gmail.com</t>
-  </si>
-  <si>
-    <t>12313132313</t>
+    <t>admin1@gmail.com</t>
+  </si>
+  <si>
+    <t>1311231232</t>
   </si>
   <si>
     <t>6-A ACHARYA KRIPLANI MARG NEAR MOTI</t>
   </si>
   <si>
-    <t>3EFFVBw9</t>
+    <t>Z3zQQL1B</t>
   </si>
   <si>
     <t>["New Release","Catalogue","Payment"]</t>

</xml_diff>